<commit_message>
agregado malla facial juanjo
</commit_message>
<xml_diff>
--- a/registro_transito.xlsx
+++ b/registro_transito.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F662"/>
+  <dimension ref="A1:F684"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21144,6 +21144,710 @@
         </is>
       </c>
     </row>
+    <row r="663">
+      <c r="A663" t="inlineStr">
+        <is>
+          <t>REG-954081</t>
+        </is>
+      </c>
+      <c r="B663" t="inlineStr">
+        <is>
+          <t>persona</t>
+        </is>
+      </c>
+      <c r="C663" t="inlineStr">
+        <is>
+          <t>femenino</t>
+        </is>
+      </c>
+      <c r="D663" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="E663" t="inlineStr">
+        <is>
+          <t>19:06:14</t>
+        </is>
+      </c>
+      <c r="F663" t="inlineStr">
+        <is>
+          <t>Cámara Principal</t>
+        </is>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" t="inlineStr">
+        <is>
+          <t>REG-903366</t>
+        </is>
+      </c>
+      <c r="B664" t="inlineStr">
+        <is>
+          <t>persona</t>
+        </is>
+      </c>
+      <c r="C664" t="inlineStr">
+        <is>
+          <t>masculino</t>
+        </is>
+      </c>
+      <c r="D664" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="E664" t="inlineStr">
+        <is>
+          <t>19:06:18</t>
+        </is>
+      </c>
+      <c r="F664" t="inlineStr">
+        <is>
+          <t>Cámara Principal</t>
+        </is>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" t="inlineStr">
+        <is>
+          <t>REG-390429</t>
+        </is>
+      </c>
+      <c r="B665" t="inlineStr">
+        <is>
+          <t>persona</t>
+        </is>
+      </c>
+      <c r="C665" t="inlineStr">
+        <is>
+          <t>masculino</t>
+        </is>
+      </c>
+      <c r="D665" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="E665" t="inlineStr">
+        <is>
+          <t>19:06:22</t>
+        </is>
+      </c>
+      <c r="F665" t="inlineStr">
+        <is>
+          <t>Cámara Principal</t>
+        </is>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" t="inlineStr">
+        <is>
+          <t>REG-954909</t>
+        </is>
+      </c>
+      <c r="B666" t="inlineStr">
+        <is>
+          <t>persona</t>
+        </is>
+      </c>
+      <c r="C666" t="inlineStr">
+        <is>
+          <t>masculino</t>
+        </is>
+      </c>
+      <c r="D666" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="E666" t="inlineStr">
+        <is>
+          <t>19:06:26</t>
+        </is>
+      </c>
+      <c r="F666" t="inlineStr">
+        <is>
+          <t>Cámara Principal</t>
+        </is>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" t="inlineStr">
+        <is>
+          <t>REG-355094</t>
+        </is>
+      </c>
+      <c r="B667" t="inlineStr">
+        <is>
+          <t>persona</t>
+        </is>
+      </c>
+      <c r="C667" t="inlineStr">
+        <is>
+          <t>masculino</t>
+        </is>
+      </c>
+      <c r="D667" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="E667" t="inlineStr">
+        <is>
+          <t>19:06:31</t>
+        </is>
+      </c>
+      <c r="F667" t="inlineStr">
+        <is>
+          <t>Cámara Principal</t>
+        </is>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" t="inlineStr">
+        <is>
+          <t>REG-388223</t>
+        </is>
+      </c>
+      <c r="B668" t="inlineStr">
+        <is>
+          <t>persona</t>
+        </is>
+      </c>
+      <c r="C668" t="inlineStr">
+        <is>
+          <t>masculino</t>
+        </is>
+      </c>
+      <c r="D668" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="E668" t="inlineStr">
+        <is>
+          <t>19:06:35</t>
+        </is>
+      </c>
+      <c r="F668" t="inlineStr">
+        <is>
+          <t>Cámara Principal</t>
+        </is>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" t="inlineStr">
+        <is>
+          <t>REG-571183</t>
+        </is>
+      </c>
+      <c r="B669" t="inlineStr">
+        <is>
+          <t>persona</t>
+        </is>
+      </c>
+      <c r="C669" t="inlineStr">
+        <is>
+          <t>masculino</t>
+        </is>
+      </c>
+      <c r="D669" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="E669" t="inlineStr">
+        <is>
+          <t>19:06:39</t>
+        </is>
+      </c>
+      <c r="F669" t="inlineStr">
+        <is>
+          <t>Cámara Principal</t>
+        </is>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" t="inlineStr">
+        <is>
+          <t>REG-796776</t>
+        </is>
+      </c>
+      <c r="B670" t="inlineStr">
+        <is>
+          <t>persona</t>
+        </is>
+      </c>
+      <c r="C670" t="inlineStr">
+        <is>
+          <t>masculino</t>
+        </is>
+      </c>
+      <c r="D670" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="E670" t="inlineStr">
+        <is>
+          <t>19:06:43</t>
+        </is>
+      </c>
+      <c r="F670" t="inlineStr">
+        <is>
+          <t>Cámara Principal</t>
+        </is>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" t="inlineStr">
+        <is>
+          <t>REG-152356</t>
+        </is>
+      </c>
+      <c r="B671" t="inlineStr">
+        <is>
+          <t>persona</t>
+        </is>
+      </c>
+      <c r="C671" t="inlineStr">
+        <is>
+          <t>masculino</t>
+        </is>
+      </c>
+      <c r="D671" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="E671" t="inlineStr">
+        <is>
+          <t>19:06:47</t>
+        </is>
+      </c>
+      <c r="F671" t="inlineStr">
+        <is>
+          <t>Cámara Principal</t>
+        </is>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" t="inlineStr">
+        <is>
+          <t>REG-697951</t>
+        </is>
+      </c>
+      <c r="B672" t="inlineStr">
+        <is>
+          <t>persona</t>
+        </is>
+      </c>
+      <c r="C672" t="inlineStr">
+        <is>
+          <t>masculino</t>
+        </is>
+      </c>
+      <c r="D672" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="E672" t="inlineStr">
+        <is>
+          <t>19:06:51</t>
+        </is>
+      </c>
+      <c r="F672" t="inlineStr">
+        <is>
+          <t>Cámara Principal</t>
+        </is>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" t="inlineStr">
+        <is>
+          <t>REG-779488</t>
+        </is>
+      </c>
+      <c r="B673" t="inlineStr">
+        <is>
+          <t>persona</t>
+        </is>
+      </c>
+      <c r="C673" t="inlineStr">
+        <is>
+          <t>masculino</t>
+        </is>
+      </c>
+      <c r="D673" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="E673" t="inlineStr">
+        <is>
+          <t>19:06:55</t>
+        </is>
+      </c>
+      <c r="F673" t="inlineStr">
+        <is>
+          <t>Cámara Principal</t>
+        </is>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" t="inlineStr">
+        <is>
+          <t>REG-241274</t>
+        </is>
+      </c>
+      <c r="B674" t="inlineStr">
+        <is>
+          <t>persona</t>
+        </is>
+      </c>
+      <c r="C674" t="inlineStr">
+        <is>
+          <t>masculino</t>
+        </is>
+      </c>
+      <c r="D674" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="E674" t="inlineStr">
+        <is>
+          <t>19:06:59</t>
+        </is>
+      </c>
+      <c r="F674" t="inlineStr">
+        <is>
+          <t>Cámara Principal</t>
+        </is>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" t="inlineStr">
+        <is>
+          <t>REG-785654</t>
+        </is>
+      </c>
+      <c r="B675" t="inlineStr">
+        <is>
+          <t>persona</t>
+        </is>
+      </c>
+      <c r="C675" t="inlineStr">
+        <is>
+          <t>masculino</t>
+        </is>
+      </c>
+      <c r="D675" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="E675" t="inlineStr">
+        <is>
+          <t>19:07:03</t>
+        </is>
+      </c>
+      <c r="F675" t="inlineStr">
+        <is>
+          <t>Cámara Principal</t>
+        </is>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" t="inlineStr">
+        <is>
+          <t>REG-727841</t>
+        </is>
+      </c>
+      <c r="B676" t="inlineStr">
+        <is>
+          <t>persona</t>
+        </is>
+      </c>
+      <c r="C676" t="inlineStr">
+        <is>
+          <t>masculino</t>
+        </is>
+      </c>
+      <c r="D676" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="E676" t="inlineStr">
+        <is>
+          <t>20:09:40</t>
+        </is>
+      </c>
+      <c r="F676" t="inlineStr">
+        <is>
+          <t>Casa JYJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" t="inlineStr">
+        <is>
+          <t>REG-677250</t>
+        </is>
+      </c>
+      <c r="B677" t="inlineStr">
+        <is>
+          <t>persona</t>
+        </is>
+      </c>
+      <c r="C677" t="inlineStr">
+        <is>
+          <t>masculino</t>
+        </is>
+      </c>
+      <c r="D677" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="E677" t="inlineStr">
+        <is>
+          <t>20:09:44</t>
+        </is>
+      </c>
+      <c r="F677" t="inlineStr">
+        <is>
+          <t>Casa JYJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" t="inlineStr">
+        <is>
+          <t>REG-663976</t>
+        </is>
+      </c>
+      <c r="B678" t="inlineStr">
+        <is>
+          <t>persona</t>
+        </is>
+      </c>
+      <c r="C678" t="inlineStr">
+        <is>
+          <t>masculino</t>
+        </is>
+      </c>
+      <c r="D678" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="E678" t="inlineStr">
+        <is>
+          <t>20:09:48</t>
+        </is>
+      </c>
+      <c r="F678" t="inlineStr">
+        <is>
+          <t>Casa JYJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" t="inlineStr">
+        <is>
+          <t>REG-289317</t>
+        </is>
+      </c>
+      <c r="B679" t="inlineStr">
+        <is>
+          <t>persona</t>
+        </is>
+      </c>
+      <c r="C679" t="inlineStr">
+        <is>
+          <t>masculino</t>
+        </is>
+      </c>
+      <c r="D679" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="E679" t="inlineStr">
+        <is>
+          <t>20:09:52</t>
+        </is>
+      </c>
+      <c r="F679" t="inlineStr">
+        <is>
+          <t>Casa JYJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" t="inlineStr">
+        <is>
+          <t>REG-430686</t>
+        </is>
+      </c>
+      <c r="B680" t="inlineStr">
+        <is>
+          <t>persona</t>
+        </is>
+      </c>
+      <c r="C680" t="inlineStr">
+        <is>
+          <t>masculino</t>
+        </is>
+      </c>
+      <c r="D680" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="E680" t="inlineStr">
+        <is>
+          <t>20:09:56</t>
+        </is>
+      </c>
+      <c r="F680" t="inlineStr">
+        <is>
+          <t>Casa JYJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" t="inlineStr">
+        <is>
+          <t>REG-887754</t>
+        </is>
+      </c>
+      <c r="B681" t="inlineStr">
+        <is>
+          <t>persona</t>
+        </is>
+      </c>
+      <c r="C681" t="inlineStr">
+        <is>
+          <t>masculino</t>
+        </is>
+      </c>
+      <c r="D681" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="E681" t="inlineStr">
+        <is>
+          <t>20:12:37</t>
+        </is>
+      </c>
+      <c r="F681" t="inlineStr">
+        <is>
+          <t>Casa JYJ</t>
+        </is>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" t="inlineStr">
+        <is>
+          <t>REG-247667</t>
+        </is>
+      </c>
+      <c r="B682" t="inlineStr">
+        <is>
+          <t>persona</t>
+        </is>
+      </c>
+      <c r="C682" t="inlineStr">
+        <is>
+          <t>femenino</t>
+        </is>
+      </c>
+      <c r="D682" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="E682" t="inlineStr">
+        <is>
+          <t>20:51:38</t>
+        </is>
+      </c>
+      <c r="F682" t="inlineStr">
+        <is>
+          <t>Casa juanjo</t>
+        </is>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" t="inlineStr">
+        <is>
+          <t>REG-637639</t>
+        </is>
+      </c>
+      <c r="B683" t="inlineStr">
+        <is>
+          <t>persona</t>
+        </is>
+      </c>
+      <c r="C683" t="inlineStr">
+        <is>
+          <t>femenino</t>
+        </is>
+      </c>
+      <c r="D683" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="E683" t="inlineStr">
+        <is>
+          <t>20:51:42</t>
+        </is>
+      </c>
+      <c r="F683" t="inlineStr">
+        <is>
+          <t>Casa juanjo</t>
+        </is>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" t="inlineStr">
+        <is>
+          <t>REG-767947</t>
+        </is>
+      </c>
+      <c r="B684" t="inlineStr">
+        <is>
+          <t>persona</t>
+        </is>
+      </c>
+      <c r="C684" t="inlineStr">
+        <is>
+          <t>masculino</t>
+        </is>
+      </c>
+      <c r="D684" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="E684" t="inlineStr">
+        <is>
+          <t>20:51:46</t>
+        </is>
+      </c>
+      <c r="F684" t="inlineStr">
+        <is>
+          <t>Casa juanjo</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Se agrego endpoint restaurado de registro de rostro
</commit_message>
<xml_diff>
--- a/registro_transito.xlsx
+++ b/registro_transito.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F751"/>
+  <dimension ref="A1:F761"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23988,6 +23988,326 @@
         </is>
       </c>
     </row>
+    <row r="752">
+      <c r="A752" t="inlineStr">
+        <is>
+          <t>REG-326519</t>
+        </is>
+      </c>
+      <c r="B752" t="inlineStr">
+        <is>
+          <t>persona</t>
+        </is>
+      </c>
+      <c r="C752" t="inlineStr">
+        <is>
+          <t>femenino</t>
+        </is>
+      </c>
+      <c r="D752" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="E752" t="inlineStr">
+        <is>
+          <t>10:56:08</t>
+        </is>
+      </c>
+      <c r="F752" t="inlineStr">
+        <is>
+          <t>Cámara Principal</t>
+        </is>
+      </c>
+    </row>
+    <row r="753">
+      <c r="A753" t="inlineStr">
+        <is>
+          <t>REG-119377</t>
+        </is>
+      </c>
+      <c r="B753" t="inlineStr">
+        <is>
+          <t>persona</t>
+        </is>
+      </c>
+      <c r="C753" t="inlineStr">
+        <is>
+          <t>masculino</t>
+        </is>
+      </c>
+      <c r="D753" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="E753" t="inlineStr">
+        <is>
+          <t>10:56:12</t>
+        </is>
+      </c>
+      <c r="F753" t="inlineStr">
+        <is>
+          <t>Cámara Principal</t>
+        </is>
+      </c>
+    </row>
+    <row r="754">
+      <c r="A754" t="inlineStr">
+        <is>
+          <t>REG-310617</t>
+        </is>
+      </c>
+      <c r="B754" t="inlineStr">
+        <is>
+          <t>persona</t>
+        </is>
+      </c>
+      <c r="C754" t="inlineStr">
+        <is>
+          <t>masculino</t>
+        </is>
+      </c>
+      <c r="D754" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="E754" t="inlineStr">
+        <is>
+          <t>10:56:16</t>
+        </is>
+      </c>
+      <c r="F754" t="inlineStr">
+        <is>
+          <t>Cámara Principal</t>
+        </is>
+      </c>
+    </row>
+    <row r="755">
+      <c r="A755" t="inlineStr">
+        <is>
+          <t>REG-226919</t>
+        </is>
+      </c>
+      <c r="B755" t="inlineStr">
+        <is>
+          <t>persona</t>
+        </is>
+      </c>
+      <c r="C755" t="inlineStr">
+        <is>
+          <t>masculino</t>
+        </is>
+      </c>
+      <c r="D755" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="E755" t="inlineStr">
+        <is>
+          <t>10:56:20</t>
+        </is>
+      </c>
+      <c r="F755" t="inlineStr">
+        <is>
+          <t>Cámara Principal</t>
+        </is>
+      </c>
+    </row>
+    <row r="756">
+      <c r="A756" t="inlineStr">
+        <is>
+          <t>REG-978836</t>
+        </is>
+      </c>
+      <c r="B756" t="inlineStr">
+        <is>
+          <t>persona</t>
+        </is>
+      </c>
+      <c r="C756" t="inlineStr">
+        <is>
+          <t>femenino</t>
+        </is>
+      </c>
+      <c r="D756" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="E756" t="inlineStr">
+        <is>
+          <t>10:56:24</t>
+        </is>
+      </c>
+      <c r="F756" t="inlineStr">
+        <is>
+          <t>Cámara Principal</t>
+        </is>
+      </c>
+    </row>
+    <row r="757">
+      <c r="A757" t="inlineStr">
+        <is>
+          <t>REG-468088</t>
+        </is>
+      </c>
+      <c r="B757" t="inlineStr">
+        <is>
+          <t>persona</t>
+        </is>
+      </c>
+      <c r="C757" t="inlineStr">
+        <is>
+          <t>masculino</t>
+        </is>
+      </c>
+      <c r="D757" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="E757" t="inlineStr">
+        <is>
+          <t>11:01:39</t>
+        </is>
+      </c>
+      <c r="F757" t="inlineStr">
+        <is>
+          <t>Cámara Principal</t>
+        </is>
+      </c>
+    </row>
+    <row r="758">
+      <c r="A758" t="inlineStr">
+        <is>
+          <t>REG-956270</t>
+        </is>
+      </c>
+      <c r="B758" t="inlineStr">
+        <is>
+          <t>persona</t>
+        </is>
+      </c>
+      <c r="C758" t="inlineStr">
+        <is>
+          <t>masculino</t>
+        </is>
+      </c>
+      <c r="D758" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="E758" t="inlineStr">
+        <is>
+          <t>11:01:43</t>
+        </is>
+      </c>
+      <c r="F758" t="inlineStr">
+        <is>
+          <t>Cámara Principal</t>
+        </is>
+      </c>
+    </row>
+    <row r="759">
+      <c r="A759" t="inlineStr">
+        <is>
+          <t>REG-930185</t>
+        </is>
+      </c>
+      <c r="B759" t="inlineStr">
+        <is>
+          <t>persona</t>
+        </is>
+      </c>
+      <c r="C759" t="inlineStr">
+        <is>
+          <t>masculino</t>
+        </is>
+      </c>
+      <c r="D759" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="E759" t="inlineStr">
+        <is>
+          <t>11:01:47</t>
+        </is>
+      </c>
+      <c r="F759" t="inlineStr">
+        <is>
+          <t>Cámara Principal</t>
+        </is>
+      </c>
+    </row>
+    <row r="760">
+      <c r="A760" t="inlineStr">
+        <is>
+          <t>REG-104154</t>
+        </is>
+      </c>
+      <c r="B760" t="inlineStr">
+        <is>
+          <t>persona</t>
+        </is>
+      </c>
+      <c r="C760" t="inlineStr">
+        <is>
+          <t>masculino</t>
+        </is>
+      </c>
+      <c r="D760" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="E760" t="inlineStr">
+        <is>
+          <t>11:01:51</t>
+        </is>
+      </c>
+      <c r="F760" t="inlineStr">
+        <is>
+          <t>Cámara Principal</t>
+        </is>
+      </c>
+    </row>
+    <row r="761">
+      <c r="A761" t="inlineStr">
+        <is>
+          <t>REG-937170</t>
+        </is>
+      </c>
+      <c r="B761" t="inlineStr">
+        <is>
+          <t>persona</t>
+        </is>
+      </c>
+      <c r="C761" t="inlineStr">
+        <is>
+          <t>masculino</t>
+        </is>
+      </c>
+      <c r="D761" t="inlineStr">
+        <is>
+          <t>2026-06-20</t>
+        </is>
+      </c>
+      <c r="E761" t="inlineStr">
+        <is>
+          <t>11:01:55</t>
+        </is>
+      </c>
+      <c r="F761" t="inlineStr">
+        <is>
+          <t>Cámara Principal</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>